<commit_message>
Improve dock reliability and team color workflow
</commit_message>
<xml_diff>
--- a/sample_sheet/PepsLive_Sheet_Template.xlsx
+++ b/sample_sheet/PepsLive_Sheet_Template.xlsx
@@ -2,8 +2,8 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Matches" sheetId="1" r:id="Rfc3ebf4a75c44a5a"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="2" r:id="R1edb5665bc0548d4"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Matches" sheetId="1" r:id="R1ffc1ba1f4cf4b4c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="2" r:id="R6c2e38bf4b4941c2"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -14,7 +14,11 @@
 
 <file path=xl/styles.xml><?xml version="1.0" encoding="utf-8"?>
 <x:styleSheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
-  <x:fonts count="4">
+  <x:numFmts count="2">
+    <x:numFmt numFmtId="200" formatCode="@"/>
+    <x:numFmt numFmtId="201" formatCode="0"/>
+  </x:numFmts>
+  <x:fonts count="5">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -22,22 +26,28 @@
     <x:font>
       <x:b/>
       <x:sz val="11"/>
-      <x:color rgb="FFFFFF"/>
+      <x:color rgb="FFFFFFFF"/>
       <x:name val="Carlito"/>
     </x:font>
     <x:font>
       <x:sz val="11"/>
-      <x:color rgb="0F172A"/>
+      <x:color rgb="FF0F172A"/>
       <x:name val="Carlito"/>
     </x:font>
     <x:font>
       <x:b/>
       <x:sz val="16"/>
-      <x:color rgb="0F172A"/>
+      <x:color rgb="FF0F172A"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="11"/>
+      <x:color rgb="FF0F172A"/>
       <x:name val="Carlito"/>
     </x:font>
   </x:fonts>
-  <x:fills count="4">
+  <x:fills count="22">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -46,12 +56,102 @@
     </x:fill>
     <x:fill>
       <x:patternFill patternType="solid">
-        <x:fgColor rgb="0F172A"/>
-      </x:patternFill>
-    </x:fill>
-    <x:fill>
-      <x:patternFill patternType="solid">
-        <x:fgColor rgb="F8FAFC"/>
+        <x:fgColor rgb="FF0F172A"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF8FAFC"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF0F172A"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFF6A00"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF111111"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF0057FF"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFFFFF"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF8FAFC"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFF4D8D"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF25121C"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF28B8FF"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF071A27"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFB000"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF18120A"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF00B894"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF071C17"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF286CFF"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF07152F"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFF3D4F"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF30080D"/>
       </x:patternFill>
     </x:fill>
   </x:fills>
@@ -62,7 +162,7 @@
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="23">
+  <x:cellXfs count="120">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -107,6 +207,217 @@
     <x:xf numFmtId="0" fontId="3" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="201" fontId="0" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="0" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="1" fillId="4" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="0" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="1" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="1" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="1" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="1" fillId="5" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="0" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="1" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="1" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="1" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="1" fillId="6" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="0" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="1" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="1" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="1" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="1" fillId="7" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="0" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="4" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="4" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="4" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="4" fillId="8" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="0" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="201" fontId="2" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="201" fontId="2" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="2" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="201" fontId="2" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="2" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="2" fillId="9" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="general" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="0" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="1" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="1" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="1" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="1" fillId="10" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="0" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="1" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="1" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="1" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="1" fillId="11" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="0" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="1" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="1" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="1" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="1" fillId="12" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="0" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="1" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="1" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="1" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="1" fillId="13" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="0" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="4" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="4" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="4" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="4" fillId="14" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="0" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="1" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="1" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="1" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="1" fillId="15" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="0" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="1" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="1" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="1" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="1" fillId="16" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="0" fillId="17" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="1" fillId="17" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="1" fillId="17" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="1" fillId="17" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="1" fillId="17" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="0" fillId="18" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="1" fillId="18" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="1" fillId="18" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="1" fillId="18" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="1" fillId="18" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="0" fillId="19" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="1" fillId="19" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="1" fillId="19" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="1" fillId="19" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="1" fillId="19" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="0" fillId="20" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="1" fillId="20" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="1" fillId="20" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="1" fillId="20" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="1" fillId="20" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="0" fillId="21" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="1" fillId="21" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="200" fontId="1" fillId="21" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="1" fillId="21" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="1" fillId="21" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="0"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -185,9 +496,9 @@
     </a:clrScheme>
     <a:fontScheme name="Office">
       <a:majorFont>
-        <a:latin typeface="Calibri"/>
-        <a:ea typeface="Calibri"/>
-        <a:cs typeface="Calibri"/>
+        <a:latin typeface="Calibri Light"/>
+        <a:ea typeface="Calibri Light"/>
+        <a:cs typeface="Calibri Light"/>
       </a:majorFont>
       <a:minorFont>
         <a:latin typeface="Calibri"/>
@@ -310,6 +621,12 @@
     <x:col min="17" max="17" width="20" hidden="0" customWidth="1"/>
     <x:col min="18" max="18" width="20" hidden="0" customWidth="1"/>
     <x:col min="19" max="19" width="20" hidden="0" customWidth="1"/>
+    <x:col min="20" max="20" width="19.3799991607666" hidden="0" customWidth="1"/>
+    <x:col min="21" max="21" width="19.3799991607666" hidden="0" customWidth="1"/>
+    <x:col min="22" max="22" width="19.3799991607666" hidden="0" customWidth="1"/>
+    <x:col min="23" max="23" width="19.3799991607666" hidden="0" customWidth="1"/>
+    <x:col min="24" max="24" width="9" hidden="0" customWidth="1"/>
+    <x:col min="25" max="25" width="21.25" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
     <x:row r="1">
@@ -369,6 +686,24 @@
       </x:c>
       <x:c r="S1" s="6" t="str">
         <x:v>Note</x:v>
+      </x:c>
+      <x:c r="T1" s="29" t="str">
+        <x:v>TeamA_PrimaryColor</x:v>
+      </x:c>
+      <x:c r="U1" s="29" t="str">
+        <x:v>TeamA_SecondaryColor</x:v>
+      </x:c>
+      <x:c r="V1" s="29" t="str">
+        <x:v>TeamB_PrimaryColor</x:v>
+      </x:c>
+      <x:c r="W1" s="29" t="str">
+        <x:v>TeamB_SecondaryColor</x:v>
+      </x:c>
+      <x:c r="X1" s="29" t="str">
+        <x:v>Revision</x:v>
+      </x:c>
+      <x:c r="Y1" s="29" t="str">
+        <x:v>LastOperationID</x:v>
       </x:c>
     </x:row>
     <x:row r="2">
@@ -411,6 +746,22 @@
       <x:c r="Q2" s="15" t="str"/>
       <x:c r="R2" s="15" t="str"/>
       <x:c r="S2" s="15" t="str"/>
+      <x:c r="T2" s="34" t="str">
+        <x:v>#FF6A00</x:v>
+      </x:c>
+      <x:c r="U2" s="39" t="str">
+        <x:v>#111111</x:v>
+      </x:c>
+      <x:c r="V2" s="44" t="str">
+        <x:v>#0057FF</x:v>
+      </x:c>
+      <x:c r="W2" s="49" t="str">
+        <x:v>#FFFFFF</x:v>
+      </x:c>
+      <x:c r="X2" s="54" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Y2" s="59"/>
     </x:row>
     <x:row r="3">
       <x:c r="A3" s="15" t="str">
@@ -452,6 +803,22 @@
       <x:c r="Q3" s="15" t="str"/>
       <x:c r="R3" s="15" t="str"/>
       <x:c r="S3" s="15" t="str"/>
+      <x:c r="T3" s="64" t="str">
+        <x:v>#FF4D8D</x:v>
+      </x:c>
+      <x:c r="U3" s="69" t="str">
+        <x:v>#25121C</x:v>
+      </x:c>
+      <x:c r="V3" s="74" t="str">
+        <x:v>#28B8FF</x:v>
+      </x:c>
+      <x:c r="W3" s="79" t="str">
+        <x:v>#071A27</x:v>
+      </x:c>
+      <x:c r="X3" s="54" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Y3" s="59"/>
     </x:row>
     <x:row r="4">
       <x:c r="A4" s="15" t="str">
@@ -493,6 +860,22 @@
       <x:c r="Q4" s="15" t="str"/>
       <x:c r="R4" s="15" t="str"/>
       <x:c r="S4" s="15" t="str"/>
+      <x:c r="T4" s="84" t="str">
+        <x:v>#FFB000</x:v>
+      </x:c>
+      <x:c r="U4" s="89" t="str">
+        <x:v>#18120A</x:v>
+      </x:c>
+      <x:c r="V4" s="94" t="str">
+        <x:v>#00B894</x:v>
+      </x:c>
+      <x:c r="W4" s="99" t="str">
+        <x:v>#071C17</x:v>
+      </x:c>
+      <x:c r="X4" s="54" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Y4" s="59"/>
     </x:row>
     <x:row r="5">
       <x:c r="A5" s="15" t="str">
@@ -534,6 +917,22 @@
       <x:c r="Q5" s="15" t="str"/>
       <x:c r="R5" s="15" t="str"/>
       <x:c r="S5" s="15" t="str"/>
+      <x:c r="T5" s="104" t="str">
+        <x:v>#286CFF</x:v>
+      </x:c>
+      <x:c r="U5" s="109" t="str">
+        <x:v>#07152F</x:v>
+      </x:c>
+      <x:c r="V5" s="114" t="str">
+        <x:v>#FF3D4F</x:v>
+      </x:c>
+      <x:c r="W5" s="119" t="str">
+        <x:v>#30080D</x:v>
+      </x:c>
+      <x:c r="X5" s="54" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="Y5" s="59"/>
     </x:row>
   </x:sheetData>
   <x:dataValidations count="1">
@@ -543,7 +942,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R432c410a649546af"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf5d82c8779894f3f"/>
   </x:tableParts>
 </x:worksheet>
 </file>

</xml_diff>

<commit_message>
Add visible Google Sheet team color sync
</commit_message>
<xml_diff>
--- a/sample_sheet/PepsLive_Sheet_Template.xlsx
+++ b/sample_sheet/PepsLive_Sheet_Template.xlsx
@@ -2,8 +2,9 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Matches" sheetId="1" r:id="R1ffc1ba1f4cf4b4c"/>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="2" r:id="R6c2e38bf4b4941c2"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Matches" sheetId="1" r:id="R6caa777faf0e404d"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="README" sheetId="2" r:id="R5d031b4d95d34b6c"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Team Colors" sheetId="3" r:id="R1bc2af9a588d45b0"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -18,7 +19,7 @@
     <x:numFmt numFmtId="200" formatCode="@"/>
     <x:numFmt numFmtId="201" formatCode="0"/>
   </x:numFmts>
-  <x:fonts count="5">
+  <x:fonts count="13">
     <x:font>
       <x:sz val="11"/>
       <x:name val="Carlito"/>
@@ -46,8 +47,50 @@
       <x:color rgb="FF0F172A"/>
       <x:name val="Carlito"/>
     </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="16"/>
+      <x:color rgb="FFFFFFFF"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:sz val="10"/>
+      <x:color rgb="FFD8E2F1"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:sz val="9"/>
+      <x:color rgb="FF93A4BA"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="10"/>
+      <x:color rgb="FFFFFFFF"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:sz val="10"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:sz val="9"/>
+      <x:color rgb="FF465568"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:b/>
+      <x:sz val="10"/>
+      <x:color rgb="FF111111"/>
+      <x:name val="Carlito"/>
+    </x:font>
+    <x:font>
+      <x:sz val="10"/>
+      <x:color rgb="FF20242B"/>
+      <x:name val="Carlito"/>
+    </x:font>
   </x:fonts>
-  <x:fills count="22">
+  <x:fills count="46">
     <x:fill>
       <x:patternFill patternType="none"/>
     </x:fill>
@@ -154,15 +197,178 @@
         <x:fgColor rgb="FF30080D"/>
       </x:patternFill>
     </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF0F172A"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF172033"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF101722"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF202A3A"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFF5F7FA"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFEEF2F7"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFF6A00"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFF4D8D"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFB000"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF286CFF"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF111111"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF25121C"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF18120A"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF07152F"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF0057FF"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF28B8FF"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF00B894"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFF3D4F"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFFFFF"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF071A27"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF071C17"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FF30080D"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFFFF2E8"/>
+      </x:patternFill>
+    </x:fill>
+    <x:fill>
+      <x:patternFill patternType="solid">
+        <x:fgColor rgb="FFEAF8F0"/>
+      </x:patternFill>
+    </x:fill>
   </x:fills>
-  <x:borders count="2">
+  <x:borders count="7">
     <x:border/>
     <x:border/>
+    <x:border>
+      <x:left style="thin">
+        <x:color rgb="FF465568"/>
+      </x:left>
+      <x:top style="thin">
+        <x:color rgb="FF465568"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FF465568"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:top style="thin">
+        <x:color rgb="FF465568"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FF465568"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:right style="thin">
+        <x:color rgb="FF465568"/>
+      </x:right>
+      <x:top style="thin">
+        <x:color rgb="FF465568"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FF465568"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:bottom style="thin">
+        <x:color rgb="FFD8DEE8"/>
+      </x:bottom>
+    </x:border>
+    <x:border>
+      <x:top style="thin">
+        <x:color rgb="FFD8DEE8"/>
+      </x:top>
+      <x:bottom style="thin">
+        <x:color rgb="FFD8DEE8"/>
+      </x:bottom>
+    </x:border>
   </x:borders>
   <x:cellStyleXfs count="1">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </x:cellStyleXfs>
-  <x:cellXfs count="120">
+  <x:cellXfs count="228">
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <x:xf numFmtId="0" fontId="0" fillId="0" borderId="1" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
     <x:xf numFmtId="0" fontId="0" fillId="2" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
@@ -418,6 +624,300 @@
     </x:xf>
     <x:xf numFmtId="200" fontId="1" fillId="21" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
       <x:alignment horizontal="center" vertical="center" wrapText="0"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="22" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="22" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="5" fillId="22" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="5" fillId="22" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="left" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="23" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="6" fillId="23" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="6" fillId="23" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="6" fillId="23" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="24" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="7" fillId="24" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="7" fillId="24" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="7" fillId="24" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="0" fillId="25" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="8" fillId="25" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="8" fillId="25" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="8" fillId="25" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="8" fillId="25" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="8" fillId="25" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="25" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="25" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="25" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="25" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="25" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="25" borderId="2" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="25" borderId="3" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="25" borderId="4" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="9" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="9" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="9" fillId="0" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="0" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="26" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="26" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="27" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="27" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="10" fillId="27" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="10" fillId="27" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="10" fillId="27" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="10" fillId="27" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="28" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="28" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="28" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="8" fillId="28" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="29" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="29" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="29" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="8" fillId="29" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="30" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="30" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="30" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="11" fillId="30" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="31" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="31" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="31" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="8" fillId="31" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="32" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="32" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="32" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="8" fillId="32" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="33" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="33" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="33" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="8" fillId="33" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="34" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="34" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="34" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="8" fillId="34" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="35" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="35" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="35" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="8" fillId="35" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="36" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="36" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="36" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="8" fillId="36" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="37" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="37" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="37" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="8" fillId="37" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="38" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="38" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="38" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="8" fillId="38" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="39" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="39" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="39" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="8" fillId="39" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="40" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="40" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="11" fillId="40" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="11" fillId="40" borderId="5" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="41" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="41" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="41" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="8" fillId="41" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="42" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="42" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="42" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="8" fillId="42" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="9" fillId="43" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="43" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="8" fillId="43" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="200" fontId="8" fillId="43" borderId="6" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment horizontal="center" vertical="center"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1"/>
+    <x:xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="0" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="44" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
+    </x:xf>
+    <x:xf numFmtId="0" fontId="12" fillId="45" borderId="0" xfId="0" applyNumberFormat="1" applyFont="1" applyFill="1" applyBorder="1" applyAlignment="1">
+      <x:alignment vertical="center" wrapText="1"/>
     </x:xf>
   </x:cellXfs>
   <x:cellStyles count="1">
@@ -450,6 +950,23 @@
     <x:tableColumn id="19" name="Note"/>
   </x:tableColumns>
   <x:tableStyleInfo name="TableStyleMedium2" showRowStripes="1"/>
+</x:table>
+</file>
+
+<file path=xl/tables/table2.xml><?xml version="1.0" encoding="utf-8"?>
+<x:table xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main" id="2" name="TeamColorsTable" displayName="TeamColorsTable" ref="A4:I8" headerRowCount="1" totalsRowCount="0" totalsRowShown="0">
+  <x:tableColumns count="9">
+    <x:tableColumn id="1" name="MatchID"/>
+    <x:tableColumn id="2" name="Team A"/>
+    <x:tableColumn id="3" name="PrimaryColor A"/>
+    <x:tableColumn id="4" name="SecondaryColor A"/>
+    <x:tableColumn id="5" name="Team B"/>
+    <x:tableColumn id="6" name="PrimaryColor B"/>
+    <x:tableColumn id="7" name="SecondaryColor B"/>
+    <x:tableColumn id="8" name="Revision"/>
+    <x:tableColumn id="9" name="Sync Status"/>
+  </x:tableColumns>
+  <x:tableStyleInfo name="TableStyleMedium2" showFirstColumn="0" showLastColumn="0" showRowStripes="1" showColumnStripes="0"/>
 </x:table>
 </file>
 
@@ -942,7 +1459,7 @@
   </x:dataValidations>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <x:tableParts count="1">
-    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf5d82c8779894f3f"/>
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="Rf0ba2d1dc8a043fa"/>
   </x:tableParts>
 </x:worksheet>
 </file>
@@ -951,45 +1468,280 @@
 <x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheetFormatPr defaultRowHeight="15"/>
   <x:cols>
-    <x:col min="1" max="1" width="110" hidden="0" customWidth="1"/>
+    <x:col min="1" max="1" width="115" hidden="0" customWidth="1"/>
   </x:cols>
   <x:sheetData>
-    <x:row r="1">
-      <x:c r="A1" s="20" t="str">
-        <x:v>PepsLive Sheet Template V1.2</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="3">
-      <x:c r="A3" s="22" t="str">
-        <x:v>ใช้ชีต Matches เป็นตารางหลัก</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="4">
-      <x:c r="A4" s="22" t="str">
-        <x:v>ห้ามลบหรือเปลี่ยนชื่อหัวตารางแถวที่ 1</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="5">
-      <x:c r="A5" s="22" t="str">
+    <x:row r="1" ht="25.5" customHeight="1">
+      <x:c r="A1" s="121" t="str">
+        <x:v>PepsLive Sheet Template V2.1</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="2">
+      <x:c r="A2" t="str"/>
+    </x:row>
+    <x:row r="3" ht="22.5" customHeight="1">
+      <x:c r="A3" s="226" t="str">
+        <x:v>เริ่มที่แท็บ Team Colors เพื่อดูสีหลักและสีรองของทั้งสองทีมได้ทันที</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="4" ht="22.5" customHeight="1">
+      <x:c r="A4" s="226" t="str">
+        <x:v>แก้ HEX ใน Team Colors หรือใช้เมนู PepsLive &gt; Pick OBS Color หลังติดตั้ง Apps Script</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5" ht="22.5" customHeight="1">
+      <x:c r="A5" s="225" t="str">
+        <x:v>ใช้ชีต Matches เป็นตารางหลักสำหรับ Dock และห้ามลบหรือเปลี่ยนชื่อหัวคอลัมน์</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6" ht="22.5" customHeight="1">
+      <x:c r="A6" s="225" t="str">
         <x:v>MatchID ต้องไม่ซ้ำ เพราะใช้สำหรับ Save Result / Finish Match กลับแถวเดิม</x:v>
       </x:c>
     </x:row>
-    <x:row r="6">
-      <x:c r="A6" s="22" t="str">
-        <x:v>Sport / TimePreset / GraphicPreset ถูกตัดออกแล้ว ให้เลือกจากหน้า PepsLive Dock</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="7">
-      <x:c r="A7" s="22" t="str">
-        <x:v>LogoA/LogoB ให้ใส่ชื่อไฟล์หรือรหัส เช่น A1 แล้ววางไฟล์ไว้ใน scoreboard/logos/A1.png</x:v>
-      </x:c>
-    </x:row>
-    <x:row r="8">
-      <x:c r="A8" s="22" t="str">
-        <x:v>หลังจบแมตช์ ระบบจะอัปเดต ScoreA, ScoreB, FinalScore, MatchStatus, Winner, FinishedAt, UpdatedAt, UpdatedBy, Note</x:v>
+    <x:row r="7" ht="22.5" customHeight="1">
+      <x:c r="A7" s="227" t="str">
+        <x:v>หลังนำเข้า Google Sheets ให้เปิด Extensions &gt; Apps Script และวางสคริปต์ล่าสุด</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8" ht="22.5" customHeight="1">
+      <x:c r="A8" s="227" t="str">
+        <x:v>Reload Sheet แล้วเลือก PepsLive &gt; Install / Repair Sheet เพื่อเปิด Team Colors sync</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="9" ht="22.5" customHeight="1">
+      <x:c r="A9" s="225" t="str">
+        <x:v>นำ URL ของ Google Sheet และ Apps Script Web App ไปใส่ในหน้า Sheet ของ Dock</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="10" ht="22.5" customHeight="1">
+      <x:c r="A10" s="225" t="str">
+        <x:v>เมื่อเตรียมสีเสร็จ ให้กด Load Sheet ใน Dock เพื่อโหลดชื่อทีม โลโก้ คะแนน และสี</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="11" ht="22.5" customHeight="1">
+      <x:c r="A11" s="225" t="str">
+        <x:v>สีใน Team Colors, Dock และ OBS Color Sources ใช้มาตรฐาน #RRGGBB เดียวกัน</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="12" ht="22.5" customHeight="1">
+      <x:c r="A12" s="225" t="str">
+        <x:v>คอลัมน์ Revision และ LastOperationID ใช้ป้องกันข้อมูลเก่าทับข้อมูลใหม่</x:v>
       </x:c>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </x:worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<x:worksheet xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+  <x:sheetFormatPr defaultRowHeight="15"/>
+  <x:cols>
+    <x:col min="1" max="1" width="11.25" hidden="0" customWidth="1"/>
+    <x:col min="2" max="2" width="22.5" hidden="0" customWidth="1"/>
+    <x:col min="3" max="3" width="15.630000114440918" hidden="0" customWidth="1"/>
+    <x:col min="4" max="4" width="16.8799991607666" hidden="0" customWidth="1"/>
+    <x:col min="5" max="5" width="22.5" hidden="0" customWidth="1"/>
+    <x:col min="6" max="6" width="15.630000114440918" hidden="0" customWidth="1"/>
+    <x:col min="7" max="7" width="16.8799991607666" hidden="0" customWidth="1"/>
+    <x:col min="8" max="8" width="9.380000114440918" hidden="0" customWidth="1"/>
+    <x:col min="9" max="9" width="22.5" hidden="0" customWidth="1"/>
+  </x:cols>
+  <x:sheetData>
+    <x:row r="1" ht="25.5" customHeight="1">
+      <x:c r="A1" s="123" t="str">
+        <x:v>TEAM COLORS | สีทีมสำหรับ PepsLive Dock + OBS</x:v>
+      </x:c>
+      <x:c r="B1" s="123"/>
+      <x:c r="C1" s="123"/>
+      <x:c r="D1" s="123"/>
+      <x:c r="E1" s="123"/>
+      <x:c r="F1" s="123"/>
+      <x:c r="G1" s="123"/>
+      <x:c r="H1" s="123"/>
+      <x:c r="I1" s="123"/>
+    </x:row>
+    <x:row r="2" ht="25.5" customHeight="1">
+      <x:c r="A2" s="127" t="str">
+        <x:v>แก้ค่า #RRGGBB ในช่องสี หรือใช้เมนู PepsLive &gt; Pick OBS Color แล้วกด Load Sheet ใน Dock</x:v>
+      </x:c>
+      <x:c r="B2" s="127"/>
+      <x:c r="C2" s="127"/>
+      <x:c r="D2" s="127"/>
+      <x:c r="E2" s="127"/>
+      <x:c r="F2" s="127"/>
+      <x:c r="G2" s="127"/>
+      <x:c r="H2" s="127"/>
+      <x:c r="I2" s="127"/>
+    </x:row>
+    <x:row r="3" ht="21" customHeight="1">
+      <x:c r="A3" s="131" t="str">
+        <x:v>หลังนำเข้า Google Sheets ให้ติดตั้ง Apps Script และใช้ PepsLive &gt; Install / Repair Sheet เพื่อเปิดการซิงก์สองทาง</x:v>
+      </x:c>
+      <x:c r="B3" s="131"/>
+      <x:c r="C3" s="131"/>
+      <x:c r="D3" s="131"/>
+      <x:c r="E3" s="131"/>
+      <x:c r="F3" s="131"/>
+      <x:c r="G3" s="131"/>
+      <x:c r="H3" s="131"/>
+      <x:c r="I3" s="131"/>
+    </x:row>
+    <x:row r="4" ht="27" customHeight="1">
+      <x:c r="A4" s="143" t="str">
+        <x:v>MatchID</x:v>
+      </x:c>
+      <x:c r="B4" s="144" t="str">
+        <x:v>Team A</x:v>
+      </x:c>
+      <x:c r="C4" s="144" t="str">
+        <x:v>PrimaryColor A</x:v>
+      </x:c>
+      <x:c r="D4" s="144" t="str">
+        <x:v>SecondaryColor A</x:v>
+      </x:c>
+      <x:c r="E4" s="144" t="str">
+        <x:v>Team B</x:v>
+      </x:c>
+      <x:c r="F4" s="144" t="str">
+        <x:v>PrimaryColor B</x:v>
+      </x:c>
+      <x:c r="G4" s="144" t="str">
+        <x:v>SecondaryColor B</x:v>
+      </x:c>
+      <x:c r="H4" s="144" t="str">
+        <x:v>Revision</x:v>
+      </x:c>
+      <x:c r="I4" s="145" t="str">
+        <x:v>Sync Status</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="5">
+      <x:c r="A5" s="151" t="str">
+        <x:v>001</x:v>
+      </x:c>
+      <x:c r="B5" s="151" t="str">
+        <x:v>ทีมบ้านเหนือ</x:v>
+      </x:c>
+      <x:c r="C5" s="162" t="str">
+        <x:v>#FF6A00</x:v>
+      </x:c>
+      <x:c r="D5" s="178" t="str">
+        <x:v>#111111</x:v>
+      </x:c>
+      <x:c r="E5" s="151" t="str">
+        <x:v>ทีมบ้านใต้</x:v>
+      </x:c>
+      <x:c r="F5" s="194" t="str">
+        <x:v>#0057FF</x:v>
+      </x:c>
+      <x:c r="G5" s="210" t="str">
+        <x:v>#FFFFFF</x:v>
+      </x:c>
+      <x:c r="H5" s="157" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I5" s="157" t="str">
+        <x:v>ติดตั้ง Apps Script เพื่อซิงก์</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="6">
+      <x:c r="A6" s="152" t="str">
+        <x:v>002</x:v>
+      </x:c>
+      <x:c r="B6" s="152" t="str">
+        <x:v>มาดามเก๋</x:v>
+      </x:c>
+      <x:c r="C6" s="166" t="str">
+        <x:v>#FF4D8D</x:v>
+      </x:c>
+      <x:c r="D6" s="182" t="str">
+        <x:v>#25121C</x:v>
+      </x:c>
+      <x:c r="E6" s="152" t="str">
+        <x:v>สุรินทร์การค้า</x:v>
+      </x:c>
+      <x:c r="F6" s="198" t="str">
+        <x:v>#28B8FF</x:v>
+      </x:c>
+      <x:c r="G6" s="214" t="str">
+        <x:v>#071A27</x:v>
+      </x:c>
+      <x:c r="H6" s="158" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I6" s="158" t="str">
+        <x:v>ติดตั้ง Apps Script เพื่อซิงก์</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="7">
+      <x:c r="A7" s="152" t="str">
+        <x:v>003</x:v>
+      </x:c>
+      <x:c r="B7" s="152" t="str">
+        <x:v>Peps Academy</x:v>
+      </x:c>
+      <x:c r="C7" s="170" t="str">
+        <x:v>#FFB000</x:v>
+      </x:c>
+      <x:c r="D7" s="186" t="str">
+        <x:v>#18120A</x:v>
+      </x:c>
+      <x:c r="E7" s="152" t="str">
+        <x:v>Sisaket United</x:v>
+      </x:c>
+      <x:c r="F7" s="202" t="str">
+        <x:v>#00B894</x:v>
+      </x:c>
+      <x:c r="G7" s="218" t="str">
+        <x:v>#071C17</x:v>
+      </x:c>
+      <x:c r="H7" s="158" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I7" s="158" t="str">
+        <x:v>ติดตั้ง Apps Script เพื่อซิงก์</x:v>
+      </x:c>
+    </x:row>
+    <x:row r="8">
+      <x:c r="A8" s="152" t="str">
+        <x:v>004</x:v>
+      </x:c>
+      <x:c r="B8" s="152" t="str">
+        <x:v>Thunder Blue</x:v>
+      </x:c>
+      <x:c r="C8" s="174" t="str">
+        <x:v>#286CFF</x:v>
+      </x:c>
+      <x:c r="D8" s="190" t="str">
+        <x:v>#07152F</x:v>
+      </x:c>
+      <x:c r="E8" s="152" t="str">
+        <x:v>Fire Red</x:v>
+      </x:c>
+      <x:c r="F8" s="206" t="str">
+        <x:v>#FF3D4F</x:v>
+      </x:c>
+      <x:c r="G8" s="222" t="str">
+        <x:v>#30080D</x:v>
+      </x:c>
+      <x:c r="H8" s="158" t="n">
+        <x:v>0</x:v>
+      </x:c>
+      <x:c r="I8" s="158" t="str">
+        <x:v>ติดตั้ง Apps Script เพื่อซิงก์</x:v>
+      </x:c>
+    </x:row>
+  </x:sheetData>
+  <x:mergeCells>
+    <x:mergeCell ref="A1:I1"/>
+    <x:mergeCell ref="A2:I2"/>
+    <x:mergeCell ref="A3:I3"/>
+  </x:mergeCells>
+  <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+  <x:tableParts count="1">
+    <x:tablePart xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" r:id="R064c5956edb7484f"/>
+  </x:tableParts>
+</x:worksheet>
 </file>
</xml_diff>